<commit_message>
data(applaud-audit): confirm 10 pilot app-map rows for first run
Verified each table's IF/EF resolution against the live ORACLE_MASTER
Application bridge (DBID + get_application steps). All 10 derived rows
correct: single IF each; EF step names match (T_BANKS_BRANCHES no-X_
asymmetry and T_AP_INVOICE_INT dual-EF confirmed); _VAL exports excluded.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBDI_to_Applaud_AppMap.xlsx
+++ b/FBDI_to_Applaud_AppMap.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="App Map" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'App Map'!$A$1:$E$1</definedName>
+  </definedNames>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +51,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -415,6 +416,13 @@
   </sheetPr>
   <dimension ref="A1:E148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="35.7109375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="53.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="72.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.7109375" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -449,9 +457,6 @@
           <t>T_ADDITIONALTRANSFERORDERCOST</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>derived</t>
@@ -481,7 +486,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -508,7 +513,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -940,7 +945,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1026,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1333,6 @@
           <t>T_DOO_ORDER_DOC_REFERENCES</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>X_T_DOO_ORDER_DOC_REFERENCES</t>
@@ -1557,7 +1561,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1588,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1642,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -1945,9 +1949,6 @@
           <t>T_FA_RETIREMENTS_T</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>derived</t>
@@ -1960,7 +1961,6 @@
           <t>T_GL_BUDGETS_INTERFACE</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>X_T_GL_BUDGETS_INTERFACE</t>
@@ -2334,7 +2334,6 @@
           <t>T_HZ_IMP_PARTYSITEUSES_T</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>X_T_HZ_IMP_PARTYSITEUSES_T</t>
@@ -2519,9 +2518,6 @@
           <t>T_INV_LPN_INTERFACE</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>derived</t>
@@ -2632,7 +2628,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2871,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2898,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2989,6 @@
           <t>T_POZ_SUP_CONTACT_ADDRESS_INT</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
           <t>X_T_POZ_SUP_CONT_ADDR</t>
@@ -3016,9 +3011,6 @@
           <t>T_POZ_SUP_THIRDPARTY_INT</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3463,7 +3455,6 @@
           <t>T_RA_CUSTOMER_BANKS_INT_ALL</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
           <t>X_T_RA_CUSTOMER_BANKS_INT_ALL; CUST_BANKS_API</t>
@@ -3648,9 +3639,6 @@
           <t>T_SAFETYSTOCKLEVEL</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3663,9 +3651,6 @@
           <t>T_SCP_EXTERNALFORECAST</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3678,9 +3663,6 @@
           <t>T_SCP_SALESORDER</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3693,9 +3675,6 @@
           <t>T_SCP_UOM_CONVERSION</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3708,9 +3687,6 @@
           <t>T_TRANSFERORDERLINES</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3912,9 +3888,6 @@
           <t>T_WO_ASSEMBLY_COMPONENT</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3927,9 +3900,6 @@
           <t>T_WO_BATCHES</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3942,9 +3912,6 @@
           <t>T_WO_HEADER</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3957,9 +3924,6 @@
           <t>T_WO_MATERIAL_LOT_NUMBERS</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3972,9 +3936,6 @@
           <t>T_WO_MATL_SERIAL_NUMBER</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
           <t>derived</t>
@@ -3987,9 +3948,6 @@
           <t>T_WO_OPERATIONS</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4002,9 +3960,6 @@
           <t>T_WO_OPERATION_MATERIALS</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4017,9 +3972,6 @@
           <t>T_WO_OPERATION_RESOURCES</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4032,9 +3984,6 @@
           <t>T_WO_OPN_RES_INSTANCES</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4047,9 +3996,6 @@
           <t>T_WO_PRODUCT_LOT_NUMBERS</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4062,9 +4008,6 @@
           <t>T_WO_SERIAL_NUMBERS</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4077,9 +4020,6 @@
           <t>T_WSH_FREIGHT_COSTS_INTERFACE</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
-      <c r="C146" t="inlineStr"/>
-      <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4092,9 +4032,6 @@
           <t>T_WSH_NEW_DEL_INTERFACE</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4107,9 +4044,6 @@
           <t>T_WSH_SHIPMENT_LINE_INTERFACE</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
           <t>derived</t>
@@ -4117,6 +4051,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>